<commit_message>
Add qualitative data and improving the README.md
</commit_message>
<xml_diff>
--- a/qualitative_analysis/codebook_Q16_pt_br.xlsx
+++ b/qualitative_analysis/codebook_Q16_pt_br.xlsx
@@ -741,7 +741,7 @@
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -762,10 +762,10 @@
     <xf borderId="0" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>